<commit_message>
Reformat xlsx: one value per column for staff manual filling
- Columns: Тип | Поле | Значение | Отметка
- Parse template lines into separate cells
- Empty fields left blank for manual entry
- Regenerate TEST device documents

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/daily-reports/TEST_DailyReport_67plus_LS67Y43279.xlsx
+++ b/equipment-templates/output/daily-reports/TEST_DailyReport_67plus_LS67Y43279.xlsx
@@ -17,17 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -50,11 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,180 +413,314 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Отметка</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Заголовок</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Текст</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>ЕЖЕДНЕВНЫЙ ОТЧЕТ О ХОДЕ ПЕРЕДАЧИ ДЕЛ</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Дата: 22.06.2026  Инженер: Александр</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>22.06.2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Инженер</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Александр</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Заголовок</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>1. ЛОКАЦИЯ ДНЯ:</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Риелторы (Тюмень)</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Локация дня</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Риелторы (Тюмень)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>2. СТАТУС ПО ОЦЕНКАМ (сводка за день):</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   🟢 Оценка 4-5 (хорошее/отличное): _____ шт.</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   🟡 Оценка 3 (удовлетворительное):   _____ шт.</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>🟢 Оценка 4-5 (хорошее/отличное):</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   🔴 Оценка 1-2 (требует внимания):   _____ шт.</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>🟡 Оценка 3 (удовлетворительное):</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>🔴 Оценка 1-2 (требует внимания):</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>3. КРАСНЫЕ ФЛАГИ (эскалация Наталье):</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   [ ] Нет</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Проверка</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   [ ] Да (кол-во: _____ шт.)</t>
-        </is>
-      </c>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Проверка</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Да (кол-во: _____ шт.)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Краткое описание:</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Краткое описание</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ___________________________________________________________</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>4. ПРОБЛЕМЫ / БЛОКЕРЫ:</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ___________________________________________________________</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Раздел</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>5. ПЛАН НА ЗАВТРА:</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Поле</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Локация</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>4. ПРОБЛЕМЫ / БЛОКЕРЫ:</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ___________________________________________________________</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ___________________________________________________________</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>5. ПЛАН НА ЗАВТРА:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Локация: _________________________________________________</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Заголовок</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
         <is>
           <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Clean xlsx layout: remove decorative lines and symbols
- Skip ═══ and ─── separator rows entirely
- Remove ☐ from Отметка column (leave blank for staff)
- Simplify to 4 columns: Поле | Значение | Ед. | Отметка

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/daily-reports/TEST_DailyReport_67plus_LS67Y43279.xlsx
+++ b/equipment-templates/output/daily-reports/TEST_DailyReport_67plus_LS67Y43279.xlsx
@@ -413,38 +413,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Поле</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Значение</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Ед.</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>Отметка</t>
         </is>
@@ -453,307 +447,174 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Заголовок</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>═══════════════════════════════════════════════════════════════</t>
-        </is>
-      </c>
+          <t>ЕЖЕДНЕВНЫЙ ОТЧЕТ О ХОДЕ ПЕРЕДАЧИ ДЕЛ</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Текст</t>
+          <t>Дата</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ЕЖЕДНЕВНЫЙ ОТЧЕТ О ХОДЕ ПЕРЕДАЧИ ДЕЛ</t>
+          <t>22.06.2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Инженер</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Дата</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>22.06.2026</t>
-        </is>
-      </c>
+          <t>Александр</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Инженер</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Александр</t>
-        </is>
-      </c>
+          <t>1. ЛОКАЦИЯ ДНЯ:</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Заголовок</t>
+          <t>Локация дня</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>═══════════════════════════════════════════════════════════════</t>
+          <t>Риелторы (Тюмень)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1. ЛОКАЦИЯ ДНЯ:</t>
-        </is>
-      </c>
+          <t>2. СТАТУС ПО ОЦЕНКАМ (сводка за день):</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Локация дня</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Риелторы (Тюмень)</t>
-        </is>
-      </c>
+          <t>🟢 Оценка 4-5 (хорошее/отличное):</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2. СТАТУС ПО ОЦЕНКАМ (сводка за день):</t>
-        </is>
-      </c>
+          <t>🟡 Оценка 3 (удовлетворительное):</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>🟢 Оценка 4-5 (хорошее/отличное):</t>
-        </is>
-      </c>
+          <t>🔴 Оценка 1-2 (требует внимания):</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>🟡 Оценка 3 (удовлетворительное):</t>
-        </is>
-      </c>
+          <t>3. КРАСНЫЕ ФЛАГИ (эскалация Наталье):</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>🔴 Оценка 1-2 (требует внимания):</t>
-        </is>
-      </c>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>3. КРАСНЫЕ ФЛАГИ (эскалация Наталье):</t>
-        </is>
-      </c>
+          <t>Да (кол-во: _____ шт.)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Проверка</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
+          <t>Краткое описание</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Проверка</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Да (кол-во: _____ шт.)</t>
-        </is>
-      </c>
+          <t>4. ПРОБЛЕМЫ / БЛОКЕРЫ:</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Краткое описание</t>
-        </is>
-      </c>
+          <t>5. ПЛАН НА ЗАВТРА:</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>4. ПРОБЛЕМЫ / БЛОКЕРЫ:</t>
-        </is>
-      </c>
+          <t>Локация</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Раздел</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>5. ПЛАН НА ЗАВТРА:</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Локация</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Заголовок</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>═══════════════════════════════════════════════════════════════</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>